<commit_message>
Update: Disease registry outputs and pipeline improvements
- Add disease registry outputs for Banana, Cauliflower, Coffee, Orange, Sugarcane, Wheat
- Update Corn, Soybean, and Tomato registry outputs with latest results
- Update pipeline.py with latest improvements
- Include discovery results, final registries, and extracted data

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/disease_registry/outputs/Corn/internet.xlsx
+++ b/disease_registry/outputs/Corn/internet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,12 +456,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Common_Rust</t>
+          <t>Anthracnose_Leaf_Spot_And_Top_Dieback</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Puccinia sorghi</t>
+          <t>Colletotrichum graminicola</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Foliar</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dark, reddish-brown pustules (uredinia) scattered over both upper and lower leaf surfaces, oval to elongate in shape, less than 1/4 inch long, surrounded by broken leaf epidermal layer. Pustules turn brownish-black as plant matures. Under severe conditions, leaf chlorosis and death may occur.. Oval to elongate dark reddish-brown pustules (uredinia) less than 1/4 inch long occurring on both the upper and lower leaf surfaces, surrounded by broken epidermis, distinguishing it from Southern rust which has pustules predominantly on the upper surface. Pustules may develop in bands across the leaf if infection occurs while leaves are in the whorl. Pustules darken to brownish-black as plant matures.. Southern rust</t>
+          <t>Oval or spindle-shaped leaf lesions with tan or brown centers and dark brown or purple margins, up to 1 inch long and ½ inch wide. Lesions can enlarge and join to blight entire leaves. As disease develops, black spiny fruiting structures appear on dead leaf tissue.. Black, spiny fruiting structures visible with a 30X hand lens on dead tissue; oval or spindle-shaped lesions with distinctive dark brown or purple margins.. Gray Leaf Spot, Eye spot</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -485,18 +485,18 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cladosporium_Ear_Rot</t>
+          <t>Anthracnose</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cladosporium herbarum</t>
+          <t>Colletotrichum graminicola</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,12 +506,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Foliar, Stem, Root, Vascular</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Dark green or black powdery mold and black streaks on kernels, with dark green or brown fuzzy mold growing on and between kernels. Mold typically forms first where kernels attach to the cob. Dark kernels scattered around the ear are also observed.. Gray to black or very dark green powdery fungal growth with black streaks in kernels; dark green fuzzy mold between kernels forming first at the kernel-cob attachment point; dark kernels scattered around the ear.</t>
+          <t>Anthracnose manifests in three phases: leaf blight with tan to brown oval lesions and black hair-like fungal structures (setae), top dieback causing stalk death above the ear, and stalk rot with shiny black discoloration and internal decay of pith and vascular tissue. In the leaf blight phase, small round to irregular water-soaked spots first appear on lower leaves, turning yellow then brown with reddish-brown borders.. Black setae (hair-like fungal structures) visible with a hand lens from necrotic leaf lesions; shiny black discoloration in blotches or streaks on lower stalk internodes that cannot be scraped off with a fingernail; shredded pith internally in stalk rot phase.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -520,20 +520,16 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Common_Smut</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Ustilago maydis</t>
-        </is>
-      </c>
+          <t>Alternaria_Black_Molds_Stem_Cankers</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Fungal</t>
@@ -541,17 +537,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Seed</t>
+          <t>Foliar, Stem, Pod</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Galls (abnormal growths) can appear anytime throughout the growing season on any above-ground plant part, including ears, leaves, stalks, or tassels. Galls are initially covered with white to silvery tissue, later developing dark masses of spores inside.. White to silvery galls on ears, leaves, stalks, or tassels that later fill with dark spore masses; leaf galls generally remain small compared to ear and stalk galls.</t>
+          <t>Black molds appear as light to dark brown lesions on the surface of ripe fruits, later covered in a black layer. Cankers appear on stems, leaves, and fruit with dark brown to black color and can lead to plant death.. Lesions vary from small flecks affecting epidermal tissue to large sunken lesions with decay extending into carpel walls. During warm, humid weather, a black velvetlike layer forms on sunken lesions.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -561,62 +557,58 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Anthracnose_Leaf_Spot_And_Top_Dieback</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Colletotrichum graminicola</t>
-        </is>
-      </c>
+          <t>Bacterial_Brown_Spot_Of_Beancanker_Of_Stone_Fruit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Foliar, Pod</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Oval or spindle-shaped tan or brown lesions with dark brown or purple margins (up to 1 inch long and ½ inch wide) beginning on lower leaves and progressing upward; lesions may enlarge up to 5–6 inches, join, and blight entire leaves. Black, spiny fruiting structures develop on dead tissue. Severely infected leaves may yellow and wither.. Black, spiny fruiting structures (acervuli with setae) visible with a 30X hand lens on dead leaf tissue; oval/spindle-shaped lesions with dark brown or purple margins. Resistant lines show only small, necrotic or chlorotic lesions.</t>
+          <t>Small brown spots on leaves that coalesce with yellowing; affected leaves develop a shot-hole appearance. Pods develop water-soaked spots that are sticky with a tiny white crusty center, eventually becoming brown and necrotic.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aspergillus_Ear_Rot</t>
+          <t>Goss_S_Wilt</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aspergillus flavus</t>
+          <t>Clavibacter michiganensis subspecies nebraskensis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Foliar, Stem, Vascular</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Olive-green to gray-green powdery mold on corn kernels, typically starting at the tip of the ear or at insect/bird/hail injury sites; spores disperse like dust when husks are pulled back. Infected kernels may appear discolored and shriveled.. Olive-green (not denim-blue) powdery mold on kernels; signs most commonly at ear tip but can be scattered throughout the ear to the base; spores disperse like dust when husk is pulled back; discolored and shriveled kernels near ear tip are associated with higher aflatoxin levels.. Penicillium ear rot</t>
+          <t>Leaves develop elongated tan lesions with irregular margins and dark water-soaked spots ('freckles'); shiny patches of dried bacterial ooze resembling dry varnish are often present on lesions; infected stalks show orange vascular bundles. Lesions can coalesce to form larger areas.. Shiny patches of dried bacterial ooze resembling dry varnish on leaf lesions; dark green to black discontinuous water-soaked spots ('freckles') within lesion margins that appear as transparent spots when observed against light; elongated tan lesions extending parallel to leaf veins; orange vascular bundles visible in infected stalks.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -631,27 +623,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Diplodia_Ear_Rot</t>
+          <t>Bacterial_Stalk_Rot</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Stenocarpella maydis</t>
+          <t>Erwinia chrysanthemi pv. zeae</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Seed, Pod</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>White fungal mycelium growing over and between kernels starting from the base of the ear. Severely affected ears turn grayish-brown, become lightweight (mummified), with rotted, soft kernels, cobs, and ear leaves. Ear leaves generally die prematurely on infected ears and husks have a bleached appearance.. Raised black bumps (pycnidia) on moldy husk or kernels; 'hidden Diplodia' shows brown kernel discoloration with pycnidia visible only when ear is broken in half. White mycelium growing from base of ear distinguishes Diplodia from Gibberella and Fusarium ear rots.. Gibberella ear rot, Fusarium ear rot</t>
+          <t>Initial discoloration of leaf sheath and stalk at nodes, progressing to lesions on leaves and sheath. Lowest internodes turn tan to brown and become water-soaked, soft, or slimy with foul odor; upper leaves wilt and soft rot occurs at the base of the whorl. The stalk rots completely and the top collapses, causing lodging.. Soft slimy rot mostly initiating at the nodes; splitting the stalk reveals internal discoloration and soft slimy rot; foul odor during decay; water-soaked soft tan-to-brown internodes.. Pythium stalk rot</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -666,12 +658,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fusarium_Disease</t>
+          <t>Aspergillus_Ear_Rot</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Fusarium verticillioides</t>
+          <t>Aspergillus flavus</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -681,12 +673,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Ear, Kernels</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Whitish to pink-colored fungal growth on kernels, often at the ear tip, sometimes with a starburst pattern of white lines radiating from a point on the kernel. Infected kernels may also be scattered on the ear.. Whitish to pink fungal growth at ear tip, and a starburst pattern appearing as white lines radiating out from a point on the kernel. Kernels can also be infected without visible symptoms.. Gibberella ear rot, Diplodia ear rot, Aspergillus ear rot</t>
+          <t>An olive-green to gray-green powdery mold appearing on corn kernels, often beginning at the ear tip and dispersing like dust when husks are pulled back; associated with discolored and shriveled kernels near the tip of the ear.. Distinctive olive-green to gray-green powdery appearance on kernels and ear; fungal spores appear powdery and disperse like dust; signs most commonly at ear tip but can be scattered throughout the ear and to the base; often associated with insect, bird, or hail injury.. Penicillium ear rot</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -695,103 +687,91 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bacterial_Stalk_Rot</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Erwinia chrysanthemi pv. zeae</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Bacterial</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Stem, Foliar, Whole plant</t>
-        </is>
-      </c>
+          <t>Penicillium_Ear_Rot</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Water-soaked, tan to brown, soft and mushy lower internodes causing sudden plant collapse, with vascular strands remaining intact; soft, brown, water-soaked rind and pith; foul odor from infected tissue; stalk twists and falls over while plant may remain green.. Water-soaked lower internodes turning tan to brown, soft and mushy; vascular strands remain intact after collapse; foul odor from infected tissue; decay at first internode above soil; stalk twists and falls over but plant may remain green because vascular tissue is not destroyed; diseased plants scattered throughout field rather than clustered.. Bacterial Top Rot, Fusarium Stalk Rot</t>
+          <t>A powdery denim-blue mold on corn ears.. Denim-blue powdery mold appearance, distinguishing it from the olive-green color of Aspergillus ear rot.. Aspergillus ear rot</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Barley_Yellow_Dwarf_Virus</t>
+          <t>Diplodia_Ear_Rot</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Barley yellow dwarf virus (BYDV)</t>
+          <t>Stenocarpella maydis and Stenocarpella macropora</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Foliar, Whole plant</t>
+          <t>Ear, Kernel, Cob, Husk</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Purpling or yellowing along leaf margins on both lower and upper leaves, with potential stunting, shorter ears, and blanking of tip ends in early infections.. Purpling or yellowing along leaf margins running the full length of leaves; color depends on variety. Distinguished from phosphate deficiency which occurs mainly on young plants.. Phosphate deficiency</t>
+          <t>White mycelium grows over and between kernels, usually starting from the base of the ear. Under highly favorable weather conditions, entire ears may become colonized, turn grayish-brown in color and lightweight (mummified), with kernels, cobs, and ear leaves that are rotted and soft.. White mycelium of the fungus growing over and between kernels, usually starting from the base of the ear — distinguishes Diplodia from Gibberella and Fusarium ear rots. Gibberella ear rot, Fusarium ear rot</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Maize_Dwarf_Mosaic_Virus</t>
+          <t>Fusarium_Disease</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Maize dwarf mosaic virus</t>
+          <t>Fusarium verticillioides</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Seed, Whole plant</t>
+          <t>Kernel, Ear</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Narrow, light green to yellow streaks along leaf veins, leaf sheaths, and husks; plants may be stunted with numerous tillers and poor seed set. Symptoms often begin as chlorotic spots and streaks on young leaves developing into mottle or mosaic patterns, with potential stunting and shortened upper internodes.. Chlorotic spots and streaks on young green leaves progressing to mottle or mosaic pattern; narrow, light green to yellow streaks along leaf veins; mosaic symptoms may disappear as temperature rises while young leaves become more yellow; shortened upper internodes and excessive tillering. Symptoms confined to whorl leaves (unlike Maize white line mosaic virus).. Ear rot, Stalk rot, Maize white line mosaic virus</t>
+          <t>White to salmon-pink discoloration of individual kernels or groups of kernels scattered over the ear. A white to pinkish weft of mycelia covers the kernels, especially on the tip of the ear. White, gray, and pink kernel streaking with starburst patterns may also be observed.. White to salmon-pink discoloration with visible mycelia covering; in severe cases ears are completely consumed, leaving lightweight husks cemented to kernels by mycelia; characteristic starburst symptoms and multi-colored streaking pattern</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -800,33 +780,33 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Corn_Stunt_Spiroplasma</t>
+          <t>Charcoal_Rot</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Spiroplasma kunkelii</t>
+          <t>Macrophomina phaseolina</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Root, Seed, Vascular, Whole plant</t>
+          <t>Root, Stem, Vascular</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Chlorosis and/or reddening of leaf tips, followed by axillary bud production, tillering, severe plant stunting due to shortened internodes, and production of multiple small ears with missing kernels.. Chlorotic stripes extending toward leaf tips, reddening of leaves, severe stunting from shortened internodes, and multiple small ears with missing kernels. Symptoms appear late in season, generally 30 days after leafhopper feeding, during reproductive stages. Severely infected plants may be only 5 feet tall with very short internodes, and stalks may bear multiple ears (up to 6-7) with loose kernels ('loose tooth ears').</t>
+          <t>Charcoal rot begins as a root infection spreading into lower stalk internodes; infected stalks become shredded with completely rotted pith leaving only stringy vascular strands intact; tiny black spherical sclerotia on the vascular strands give the internal stalk tissue a gray/charred appearance; upper leaves dry out; plants wilt.. Small, black, spherical sclerotia of the fungus found on and in vascular strands, numerous enough to give internal stalk tissue a gray color; pith is completely rotted while stringy vascular strands remain more or less intact.. Insufficient water stress, Bacterial wilt, Root problems</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -835,33 +815,33 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Crazy_Top</t>
+          <t>Carbonum_Leaf_Spot</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sclerophthora macrospora</t>
+          <t>Cochliobolus carbonum</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Oomycete</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Whole plant</t>
+          <t>Foliar</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Plants are distorted and/or stunted with a bushy appearance at the top due to leaf proliferation below the tassel, shortened or elongated internodes, excessive tillering, narrow strap-like leaves, and possible lack of ear and tassel formation.. Proliferation of leaves below the tassel giving a very bushy appearance to the top of the plant, excessive tillering, narrow strap-like leaves, and shortened internodes.</t>
+          <t>Symptoms typically appear at silking or full maturity, consisting of circular tan to brown lesions (1/8 to ½ inch) running in a line along the leaf vein.. Lesions arranged in a linear pattern along leaf veins, often described as looking like a 'string of pearls.'</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -876,43 +856,47 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Damping_Off</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t>Barley_Yellow_Dwarf_Virus</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Barley yellow dwarf virus (BYDV)</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Stem, Seed, Whole plant</t>
+          <t>Foliar, Whole plant</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Corn seedlings are stunted compared to healthy seedlings, with a rotted mesocotyl. Affected seedlings occur in areas with heavier, wetter soil.. Rotted mesocotyl on stunted seedlings; the mesocotyl should normally remain firm and white through at least growth stage V6.. Anhydrous ammonia injury, Wireworm damage, Cold injury</t>
+          <t>Symptoms appear as faint yellowish-green blotches near the leaf tip that enlarge and merge, changing to red-purple in oats, yellow-red in wheat, and bright yellow in barley. Infected plants are dwarfed with leaves becoming stiff and erect.. Reddish-purple or yellowish discoloration of the flag leaf combined with plant dwarfing. Symptom color varies by host: red-purple in oats, yellow-red in wheat, bright yellow in barley. Also presents with upright, stiff leaves with serrated edges, reduced tillering and flowering, and sterility with fewer, smaller kernels.. mineral deficiencies, low temperature damage, root rots, herbicide injury</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Diplodia_Stalk_Rot</t>
+          <t>Physoderma_Brown_Spot</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Stenocarpella maydis</t>
+          <t>Physoderma maydis</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -922,47 +906,47 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Stem</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Small black structures embedded within the lower stalk rind, with tan to brown discoloration of macerated pith in lower nodes.. Small black structures embedded within lower stalk rind, distinguishing it from the shiny black areas of anthracnose or the pinhead structures of charcoal rot.. Anthracnose stalk rot, Charcoal rot, Gibberella stalk rot, Fusarium stalk rot</t>
+          <t>Lesions appear on mid-canopy leaves and stalks as dark purple to black discolorations, with banding of yellowish-brown lesions across leaves.. Dark purple to black lesions on stalks and midrib with banding patterns of yellowish-brown lesions across leaves.. Septoria brown spot</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Carbonum_Leaf_Spot</t>
+          <t>Holcus_Spot</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bipolaris zeicola</t>
+          <t>Pseudomonas syringae pv. syringae</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Foliar, Leaf sheath, Husk</t>
+          <t>Foliar</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Circular tan to brown lesions (1/8 to 1/2 inch) running in a line along the leaf vein, often described as looking like a "string of pearls." Also described as grayish tan lesions surrounded by a darker border on lower leaf blades, narrow and up to 1 inch long. Symptoms usually appear at the time of silking or full maturity.. Circular tan to brown lesions arranged in a line along the leaf vein, resembling a "string of pearls". Race 2 produces oblong lesions mainly on lower leaves and on maturing plants. Race 3 produces narrow, linear lesions on leaves, leaf sheaths, and sometimes husks.. Northern Corn Leaf Blight, Southern Corn Leaf Blight, Anthracnose, Gray Leaf Spot</t>
+          <t>Water-soaked, dark green lesions initially appear near leaf tips, developing into round or elliptical tan to white spots with red to brown margins and yellow halos.. Round or elliptical tan to white spots 1/8 to 1/4 inch in diameter with red to brown margins that may be surrounded by yellow halos; spots lack margins typical of eyespot and do not necessarily develop on lower leaves first.. Paraquat damage, eyespot, gray leaf spot</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -971,18 +955,18 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Gibberella_Disease</t>
+          <t>Cladosporium_Ear_Rot</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fusarium graminearum</t>
+          <t>Cladosporium herbarum</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -997,27 +981,27 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Red or pink colored mold on corn ears, almost always beginning at the tip of the ear. In severe cases, pink mold is visible on the outside of the husks at the ear tip. Excessive mold may cause silks and husks to adhere to the ear.. Red or pink mold starting at the ear tip; infection via the silk channel; excessive mold causing silks and husks to adhere to the ear; pinkish-white mold at the tip.. Fusarium Kernel or Ear Rot</t>
+          <t>Dark (brown to green) fuzzy mold grows on and between kernels, with dark kernels scattered around the ear.. Gray to black or very dark green fungus with a powdery appearance; also causes black streaks in the kernels.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nigrospora_Ear_Rot</t>
+          <t>Common_Rust</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nigrospora oryzae</t>
+          <t>Puccinia sorghi</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1027,32 +1011,32 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Gray fungal growth on corn kernels with small black spores. Corn cobs prone to shredding during shelling.. Small black spores that can be removed by rubbing with a finger, unlike the pycnidia of Diplodia ear rot. Gray fungal growth on kernels.. Diplodia Ear Rot</t>
+          <t>Common rust begins with small tan spots on leaves with a characteristic yellow halo, progressing to brick-red to cinnamon-brown pustules that readily rub off onto fingers.. Characteristic yellow halo with jagged, elongate, brick-red to cinnamon-brown pustules that readily rub off; as disease progresses, darker orange-brown teliospores create darker pustules.. Gray leaf spot</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Penicillium_Ear_Rot</t>
+          <t>Eyespot</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Penicillium spp.</t>
+          <t>Aureobasidium zeae (synonym: Kabatiella zeae)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1062,12 +1046,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Kernel, Ear tip</t>
+          <t>Leaf, Leaf sheath, Husk</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Green or blue-green powdery mold growing between kernels, usually at the tip of the ear. Infected kernels can appear bleached or streaked.. Green or blue-green powdery mold between kernels, typically at ear tip; bleached or streaked kernels; 'blue-eye' condition (embryo discoloration) in stored grain at high moisture.</t>
+          <t>Initial symptoms are small, circular water-soaked or chlorotic spots (1/16 to 1/8 inch diameter) with yellow halos. The center tissue dies and turns tan-colored with a brown to purple ring at the margin. The yellow halo is clearly visible when the leaf is lighted from behind. Spots may coalesce into large necrotic areas and entire leaves may die.. Yellow halo clearly visible when the leaf is lighted from behind, surrounding a tan-colored necrotic center with a brown ring at the margin. Physiological leaf spot, Genetic leaf spot</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1082,47 +1066,35 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Trichoderma_Ear_Rot</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Trichoderma afroharzianum</t>
-        </is>
-      </c>
+          <t>Gray_Leaf_Spot</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>Fungal</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Seed, Husk</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>White mycelium growing between kernels and on husk leaves, with massive production of green to gray-green conidia, often covering the entire ear and causing premature ripening of kernels. Kernels may sprout on the cob if disease is severe.. Dark blue-green layers of conidia on and between kernels; white mycelium on husk leaves turning green to gray-green; premature germination/ripening of kernels; symptoms typically occurring from base to middle of cob covering all kernels and husk leaf layers.. Fusarium ear rot</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Charcoal_Stalk_Rot</t>
+          <t>Crown_Rot</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Macrophomina phaseolina</t>
+          <t>Alternaria linariae</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1132,17 +1104,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Root, Stem, Vascular</t>
+          <t>Stem</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Shredded stalks with rotted pith leaving only stringy vascular strands, covered in tiny black spherical sclerotia that give the internal stalk tissue a grey or charred appearance. Upper leaves dry out and plants ripen prematurely.. Very tiny black sclerotia on the vascular strands of the shredded pith giving a charred appearance inside the stalk. This charring of the interior is the distinguishing characteristic.. Diplodia Stalk Rot, Gibberella Stalk Rot</t>
+          <t>In seedlings, collar rot stem lesions are small, dark, and slightly sunken, forming circular or elongated lesions with or without pronounced concentric rings and light centers. Once planted in the field, lesions enlarge around the stem and girdle plants, often causing plant death or severe reduction in growth and yield.. Concentric rings may not always be pronounced, in contrast to Alternaria stem canker which always displays pronounced concentric rings.. Alternaria stem canker</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1152,12 +1124,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Northern_Leaf_Blight</t>
+          <t>Gibberella_Disease</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Exserohilum turcicum</t>
+          <t>Fusarium graminearum</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1167,12 +1139,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Foliar</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Canoe- or cigar-shaped tan to gray lesions 1 to 6 inches long on leaves, initially bordered by gray-green margins. Early lesions appear as small light-green to grayish spots. As disease develops, lesions produce dark gray spores giving a dirty appearance. Severely affected leaves become grayish-green and brittle.. Cigar- or canoe-shaped gray to tan lesions 1–6 inches long; early lesions appear as small light-green to grayish spots 1–2 weeks after infection; mature lesions produce dark gray spores giving a dirty appearance; severely affected leaves become grayish-green and brittle, resembling frost-killed leaves.. Goss's leaf blight, Stewart's wilt</t>
+          <t>GER is characterized by a pink to reddish mold that appears at the tip and grows down the ear. In early ear infection by the disease the entire ear may rot and be covered with a pinkish mycelium that causes the husk to tightly adhere to the ear. Also called red rot, infection is characterized by reddish-pinkish color of infected ears.. Pink to reddish mold progressing from tip down the ear; pinkish mycelium covering the ear causing husk to adhere tightly; blue or black perithecia may cover husk and ear shanks; pinkish-whitish mycelia visible on infected kernels.. Fusarium ear rot</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1181,18 +1153,18 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gray_Leaf_Spot</t>
+          <t>Trichoderma_Ear_Rot</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cercospora zeae-maydis</t>
+          <t>Trichoderma viride</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1202,17 +1174,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Seed, Pod</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Rectangular tan to brown lesions bordered by leaf veins, initially yellow to tan with a faint watery halo, later developing a silvery-gray cast when conidia are produced.. Rectangular lesions bordered by leaf veins, 3 to 4 inches long and 1/16 to 1/8 inch wide, with a silvery-gray cast during sporulation. Early lesions have a faint watery halo visible when held to light.. Anthracnose leaf blight, Bacterial leaf streak, Common rust, Curvularia leaf spot, Eyespot of Corn, Northern corn leaf blight, Southern corn leaf blight</t>
+          <t>Dark green mold growing on or between kernels, often covering the entire ear. Kernels may sprout on the cob if disease is severe.. Dark green mold appearing on or between kernels and covering the entire ear.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1222,27 +1194,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Downy_Mildew</t>
+          <t>Southern_Rust</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Peronosclerospora sorghi</t>
+          <t>Puccinia polysora</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Oomycete</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Foliar, Whole plant, Seed</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Leaves show yellow to white stripes from base toward tip; plants may be stunted, chlorotic, with irregular seed set. Infected leaves are narrower than usual, erect, and shredded.. Yellow to white striping on leaves from base toward tip, leaves narrower than usual, erect and shredded, white downy mycelium on both leaf surfaces.</t>
+          <t>Southern corn rust begins with small circular-to-oval lesions with light green to yellow halos, developing into light orange to cinnamon-red pustules that are smaller, more circular, and more densely packed than common rust pustules.. Smaller and more circular pustules that are densely packed; almost exclusively located on upper leaf surface; can also develop on stalk, husk, and leaf sheath unlike common rust.. Gray leaf spot</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1257,12 +1229,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Eyespot</t>
+          <t>Common_Smut</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aureobasidium zeae</t>
+          <t>Ustilago maydis</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1272,32 +1244,32 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Foliar</t>
+          <t>Foliar, Stem, Pod</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Small circular water-soaked spots with yellow halos on leaves that develop into tan spots surrounded by brown to purple rings with narrow yellow halos. Spots can join together to form large necrotic areas.. Tan spot surrounded by a brown to purple ring and narrow yellow halo, forming a characteristic 'eyespot' pattern. Lesions can also develop on leaf sheaths and husks.. physiological leaf spot, genetic leaf spot</t>
+          <t>Common smut causes yellowing of green tissue and production of light green or white to gray, fleshy galls on leaves, tassels, stalks and ears, ranging from 0.2 inches on leaves to up to 6 inches on stalks and ears. Galls are filled with black, powdery teliospores that are released when galls rupture.. Galls filled with black, powdery teliospores that rupture to release spores; galls appear light green or white to gray and fleshy; lumpy and mushroom-like in appearance with off-white to grey color, filling with fine black spores.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Crown_Rot</t>
+          <t>Head_Smut</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fusarium spp.</t>
+          <t>Sporisorium reilianum</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1307,12 +1279,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Root, Stem, Foliar, Whole plant</t>
+          <t>Tassel, Ear, Leaf, Vascular</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Stunted, wilted plants with yellowed lower leaves; brown to black discoloration of crown tissue and roots; premature senescence with grayish-green discoloration ('ghost' plants); pinkish or reddish brace roots. Stalk nodes appear reddish-brown to dark black; leaf firing starts from plant base and progresses upward.. Dark brown to black discoloration of crown interior and roots; stalk nodes rot progressively up the stalk but internodes are not typically symptomatic; distinguishable from red root rot by dark brown-black (vs. deep red-purple) discoloration. Dark discoloration visible as early as 2-leaf stage.. Red root rot, Fusarium stalk rot, Root rot</t>
+          <t>Head smut is characterized by large smut galls that replace ears or tassels, first covered by fragile, creamy white membranes that eventually rupture to release masses of dark brown spores. Sporulating fungal sites may also appear on leaves, with coarse galls revealing dry spore masses with visible strands of vascular tissue.. The vascular bundles within the galls readily differentiate head smut from common smut, giving the spore masses a stringy appearance. The gall is coarse and on eruption reveals dry spore masses with strands of vascular tissue.. common smut</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1327,49 +1299,45 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rhizoctonia</t>
+          <t>Crazy_Top</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rhizoctonia solani</t>
+          <t>Sclerophthora macrospora</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Oomycete</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Root, Stem, Whole plant</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Reddish-brown lesions on the lower stem at soil level. In corn, seedlings may die and rot below the soil surface, characterized by water-soaked and dark mesocotyl tissue that can be removed to reveal white inner vascular tissue. Also causes damping off, stem rot, root rot, crown rot, aerial web blighting, wilting, and stunting.. Reddish-brown lesions on the lower stem at soil level; in corn, water-soaked dark mesocotyl tissue removable to reveal white inner vascular tissue; girdling lesions at the soil line; small brown sclerotia may be present.. Pythium seedling disease, Fusarium root rot, Phytophthora root rot</t>
+          <t>The disease causes proliferation of the tassel where leafy structures develop instead of a normal tassel, along with abnormal tillers and chlorotic striping on leaves.. Proliferation of the tassel with a mass of leafy structures developing instead of a normal tassel structure.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Physoderma_Brown_Spot</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Physoderma maydis</t>
-        </is>
-      </c>
+          <t>Damping_Off</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Fungal</t>
@@ -1377,74 +1345,82 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Numerous very small round or oval yellowish to brown spots occurring in broad bands across the leaf, with dark purplish to black oval spots on the midrib, stalk, leaf sheath, and husks. As disease progresses, lesions coalesce and darken to chocolate, reddish brown, or purple.. Lesions develop in distinct bands across the leaf, particularly at the base. On the leaf midrib, lesions are darker and sometimes larger. Purplish to black oval spots on the midrib are filled with thousands of sporangia. Lesions are not rust pustules under magnification.. Southern Rust, Eyespot, Purple leaf sheath</t>
+          <t>Diseased corn seedlings are stunted with a rotted mesocotyl.. A rotted mesocotyl where it should normally remain firm and white.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>General_And_Mixed_Stalk_Rots</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
+          <t>Downy_Mildew</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Peronosporaceae spp. (oomycetes)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Oomycete</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Stem, Vascular</t>
+          <t>Foliar, Stem, Root, Seed, Whole plant</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Weakened stalks that are susceptible to lodging before harvest, with reduced ability to transport water and nutrients.</t>
+          <t>Characteristic symptoms include development of chlorotic streaks on leaves with stunted and bushy plant appearance due to shortened internodes, and white downy growth visible on the lower leaf surface.. White downy growth on the lower surface of leaves consisting of sporangiophores bearing hyaline, oblong or ovoid sporangia; downy growth also appears on bracts of unopened male flowers in the tassel; proliferation of axillary buds on stalk and cobs.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pythium_Stalk_Rot</t>
+          <t>Northern_Leaf_Blight</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pythium aphanidermatum</t>
+          <t>Exserohilum turcicum</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Oomycete</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Stem</t>
+          <t>Foliar, Leaf sheaths, Ear husks</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Plants suddenly fall over with dark brown, water-soaked, soft, and collapsed areas on a single internode near the soil line. The rind and pith become soft, brown, and water-soaked. Stalks may be twisted and distorted, but plants remain green and turgid briefly after collapse because the vascular tissue is not destroyed.. Infected plants remain green and turgid for a short time after collapse because the vascular bundles remain intact, distinguishing it from other stalk rots where wilting occurs simultaneously. Decay localized to the first internode above the soil; rind and pith become soft, brown, and water-soaked; stalk twists and falls over.. Anthracnose Stalk Rot, Bacterial Stalk Rot, Diplodia Stalk Rot, Fusarium Stalk Rot, Gibberella Crown Rot and Stalk Rot, Physoderma Stalk Rot</t>
+          <t>Characteristic cigar-shaped gray- to tan-colored lesions on corn leaves that initially appear as small light-green to grayish spots and develop dark gray spores, eventually destroying leaves and causing them to become grayish-green and brittle. Early symptoms appear as long, narrow tan lesions running parallel to leaf veins that expand to form long, oblong, or cigar-shaped tan to gray lesions.. One-to-six inch long cigar-shaped gray to tan lesions; compatible interactions produce large necrotic cigar-shaped lesions while incompatible interactions produce small chlorotic lesions. Lesions eventually coalesce and may cover a significant portion of the leaf, with small fungal spores appearing as tiny black or dark green specks inside lesions when observed with a hand lens.. Gray leaf spot</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1459,62 +1435,62 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Head_Smut</t>
+          <t>Maize_Chlorotic_Dwarf_Virus</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sphacelotheca reiliana</t>
+          <t>Maize chlorotic dwarf virus</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Tassel, Ear, Whole plant</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Large smut galls replace ears or tassels, first covered by fragile creamy white membranes that rupture to release masses of dark brown spores. Leaf-like proliferations develop on tassels and ears; infected ears are teardrop-shaped and lack silks. Plants may be severely dwarfed.. Intact threadlike strands of vascular bundles within spore masses give a stringy appearance, differentiating head smut from common smut. Teardrop-shaped ears lacking silks with husks filled with teliospores. Plants are systemically infected as seedlings though symptoms are only obvious at flowering.. Common smut</t>
+          <t>MCDV causes plant stunting, leaf reddening or yellowing, leaf twisting and tearing, and chlorosis of leaf veins (vein banding). Infected leaves may develop a rough corduroy texture.. Vein banding (chlorosis of leaf veins) is the most diagnostic symptom. Infected leaves develop a rough corduroy texture instead of smooth and shiny appearance.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Southern_Corn_Leaf_Blight</t>
+          <t>Maize_Dwarf_Mosaic_Virus</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Bipolaris maydis</t>
+          <t>Maize dwarf mosaic virus</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Seed</t>
+          <t>Foliar, Stem, Whole plant</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tan, rectangular lesions with reddish-brown margins on leaves (Race O); rectangular to elliptical lesions with reddish-brown border and chlorotic zone on leaves, purple spots with tan-gray centers on stalks, and gray-black felt-like mold on ears (Race T).. Rectangular spots confined by leaf veins, light brown with darker brown margin, starting on lower leaves, oval at first becoming rectangular up to 2.5 cm long and 2-6 mm wide; Race T lesions rectangular to elliptical with reddish-brown border surrounded by a chlorotic zone; stalk infections as purple spots developing tan-gray centers; ear infections as gray-black felt-like mold extending from husk into kernels.</t>
+          <t>Symptoms include narrow, light green to yellow streaks along veins of leaves and husks that may disappear with temperature rise, while young leaves become more yellow. Symptoms often begin as chlorotic spots and streaks on young leaves developing into a mottle or mosaic pattern. Plants may be stunted with numerous tillers and poor seed set.. Narrow, light green to yellow streaks along leaf veins and husks transitioning to yellow leaves as temperature increases; chlorotic spots and streaks on young leaves progressing to mosaic or mottle pattern; shortened upper internodes; excessive tillering.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1529,62 +1505,54 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Holcus_Spot</t>
+          <t>Maize_White_Line_Mosaic</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pseudomonas syringae pv. syringae</t>
+          <t>Aureusvirus zeae</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bacterial</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Foliar</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Circular, oval, or irregular dark green water-soaked spots that dry to light tan or white with papery texture, often developing light brown to reddish margins surrounded by yellow halos. Spots range from 1/8 to 1/4 inch in diameter and appear randomly across the leaf surface, especially on the upper half of leaves and near tips of lower leaves.. Spots are larger than a pencil eraser tip, lesion patterns vary leaf to leaf, water-soaked margins are present, and symptoms do not follow a clear gradient across the field. Lesions are randomly distributed with tan centers and reddish-brown margins or yellow halos. Round or elliptical tan to white spots 1/8 to 1/4 inch in diameter with red to brown margins and yellow halos.. Contact herbicide injury (paraquat), Eyespot, Gray Leaf Spot, Tar Spot</t>
-        </is>
-      </c>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Goss_S_Wilt</t>
+          <t>Nigrospora_Ear_Rot</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Clavibacter michiganensis subsp. nebraskensis</t>
+          <t>Nigrospora oryzae</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Foliar, Vascular, Stem, Whole plant</t>
+          <t>Seed, Cob</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Long, gray-green to black, water-soaked leaf lesions with wavy edges containing distinctive dark freckle-like streaks; bacterial exudate droplets dry into crystalline deposits on the leaf surface. Systemically infected plants may show discolored vascular tissue and slimy stalk rot.. Dark freckle-like streaks within lesions that are transparent when held to light, with crystalline deposits from dried bacterial exudate on the leaf surface. Lesions have distinctive wavy edges. Freckles appear as dark green to black discontinuous water-soaked spots near the edges of expanding lesions.</t>
+          <t>Nigrospora ear and cob rot displays dark gray or black fungal mold and small black spores on kernels, which become bleached with white streaks, while cobs develop a brown tattered appearance and infected ears become lighter with loose kernels. Symptoms are not usually evident until harvest; affected ears are lightweight with the cob shredding easily.. Dark gray or black mold is characteristic of this disease; numerous round black spores form at the tip end of the ear; cob shreds easily, usually at the base of the ear.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1599,97 +1567,97 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Root_Rot</t>
+          <t>Stewart_S_Wilt</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fusarium spp.</t>
+          <t>Pantoea stewartii subsp. stewartii</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Root</t>
+          <t>Foliar, Vascular, Stem, Whole plant</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Dark brown to black, discolored decaying or completely rotted roots.. Dark brown to black discolored decaying or completely rotted roots with complex symptoms.</t>
+          <t>Stewart's wilt exhibits two phases: a seedling wilt phase with water-soaked lesions and rapid wilting, and a leaf blight phase with long linear yellow-grey streaks with wavy margins running parallel to leaf veins, later turning necrotic and dark. Gray-green to yellow-green lesions may cause entire leaves to become straw-colored and necrotic.. Long linear yellow-grey lesions with wavy margins running parallel to leaf veins; water-soaked lesions progressing to necrosis; yellow bacterial slime exuding from vascular bundles in cross-sectional stem cuts; distinct wilt vs. leaf blight phase depending on plant developmental stage at infection.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Maize_Chlorotic_Dwarf_Virus</t>
+          <t>Penicillium_On_Seedling</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Maize chlorotic dwarf virus</t>
+          <t>Penicillium spp.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Foliar, Whole plant</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Plant stunting with shortening of upper internodes, leaf reddening or yellowing, leaf twisting and tearing, chlorosis of leaf veins (vein banding), and a rough "corduroy" texture on infected leaves.. Vein banding (chlorosis or clearing of the smallest visible leaf veins) is the most diagnostic symptom. Leaves may also develop a rough "corduroy" texture instead of being smooth and shiny.. Maize Dwarf Mosaic Virus</t>
+          <t>Seedlings become blighted one to two weeks after emergence with marginal scorching and dying. Green fungal growth is visible in the hypocotyl area immediately above the seed.. Green fungal growth associated with rotted areas on the hypocotyl immediately above the seed.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Maize_White_Line_Mosaic</t>
+          <t>Physoderma_Stalk_Rot</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Maize white line mosaic virus</t>
+          <t>Physoderma maydis</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Foliar, Root, Seed, Whole plant</t>
+          <t>Stem</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Severely stunted plants with bright mosaic on leaves consisting of white, yellow and yellow-green rectangular to linear patches and stripes. Cobs do not fill out, are mis-shapen and contain few kernels.. Symptoms are not confined to whorl leaves (unlike Maize dwarf mosaic virus) but are present in all leaves and persist after pollination. White line and mosaic patterns with rectangular to linear (1-2 cm) patches are distinctive. No other virus known in maize gives symptoms like those of Maize white line mosaic virus.. Maize dwarf mosaic virus</t>
+          <t>Symptoms appear when plants break at the first or second node, which becomes black with some pith rot. Infected nodes snap easily when gently pushed.. Microscopic examination reveals thousands of light brown sporangia where spore production and storage occurs. Infected nodes snap easily when gently pushed.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1704,183 +1672,159 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Physoderma_Stalk_Rot</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Physoderma maydis</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Fungal</t>
-        </is>
-      </c>
+          <t>Purple_Leaf_Sheath</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Stem</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Plants break at the first or second node, with black nodes and pith rot present. Infected nodes snap easily if gently pushed. Affected plants often look healthy with no visible brown spot symptoms on leaves.. Black nodes at first or second node, pith rot, nodes that snap easily when pushed, and microscopic light brown sporangia in symptomatic tissue. Brown spot symptoms often are not visible on the leaves of affected plants.. Anthracnose Stalk Rot of Corn, Fusarium Stalk Rot of Corn, Pythium Stalk Rot of Corn, Gibberella Crown Rot and Stalk Rot of Corn, Bacterial Stalk Rot of Corn, Diplodia Stalk Rot of Corn</t>
+          <t>Dark lesions on corn stalks and leaf collars that vary in color from purple to brown to black, typically appearing after the VT tasseling stage.. Lesions appear scattered and random across plants, with tassel debris typically present in the leaf collar area where symptoms develop.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Purple_Leaf_Sheath</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
+          <t>Pythium_Root_And_Stem_Rot</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Pythium spp.</t>
+        </is>
+      </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Abiotic</t>
+          <t>Oomycete</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Stem, Foliar</t>
+          <t>Seed, Root, Stem</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Dark lesions on corn stalks and leaf collars, with color varying from purple to brown to black. Affected plants are scattered and random throughout the field.. Pieces of tassel debris fallen into the leaf collar are present in almost all cases where symptoms appear; lesions are not specific to any hybrid, canopy position, or field location and affected plants are scattered randomly.</t>
+          <t>Symptoms range from stunted, slower-growing plants to severely infected, dead plants, with brown, rotted roots and necrotic mesocotyl. Typical symptoms include seed decay, pre-emergent seedling rot, and seedling damping off. If the plant has emerged, the root system's outer layer can be easily pulled off while the center stays intact; dark lesions may develop on the mesocotyl or root system in corn.. Root system where the outer layer can be easily pulled off with the center remaining intact (rat tail-like appearance); dark lesions on mesocotyl or root system in corn; brown rotted roots and mesocotyl.. Rhizoctonia Root Rot, Fusarium Root Rot, Phytophthora, Insect injury, Herbicide damage</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pythium</t>
+          <t>Common_Corn_Rust</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Pythium spp.</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Oomycete</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Root, Seed, Stem</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Dark, slimy, water-soaked lesions on roots and mesocotyl that cause shriveling. The outer cortex of the root may rot while the inner stele remains white and intact.. Water-soaked appearance of infected tissue; outer root cortex rots while the inner stele remains white and intact; dark, slimy lesions on root or mesocotyl. Most favored by wet/saturated soil conditions due to production of motile swimming zoospores.. Fusarium seedling blight and root rot, Rhizoctonia seedling blight and root rot, Penicillium seedling blight</t>
-        </is>
-      </c>
+          <t>Puccinia polysora</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Stewart_S_Disease</t>
+          <t>Southern_Corn_Leaf_Blight</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pantoea stewartii</t>
+          <t>Bipolaris maydis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Foliar, Vascular, Stem, Whole plant</t>
+          <t>Foliar, Stem, Pod, Seed</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Bleached leaf streaks running the length of the leaf in early phase, progressing to leaf blight after tasseling; internal vascular discoloration and bacterial oozing from cut stems; seedlings may wilt and die when severe.. Bleached leaf streaks that may run the full length of the leaf; bacterial oozing from cut stem cross sections; discoloration of vascular tissues; two distinct phases with early seedling wilt and later leaf blight after tasseling.. Goss's Wilt</t>
+          <t>Two races cause distinct lesion patterns. Race O produces tan lesions with reddish-brown margins on leaves; Race T produces reddish-brown margined lesions with possible chlorotic zones. Stalk infections show purple spots with tan-gray centers, and ear infections display gray-black lesions extending into kernels with black felt-like mold.. Race O distinctly produces tan lesions with reddish-brown margins and rectangular shape; Race T produces reddish-brown margined lesions rectangular to elliptical in shape (1/4 to 1/2 inch wide by 1/4 to 3/4 inch long) possibly surrounded by a chlorotic zone. Stalk infections appear as purple spots developing tan-gray centers. Ear infections show gray-black lesions with black felt-like mold extending into kernels.. Northern corn leaf blight, Northern corn leaf spot</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Southern_Rust</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Puccinia polysora</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Fungal</t>
-        </is>
-      </c>
+          <t>Root_Rot</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Root</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Small circular-to-oval shaped lesions with light green to yellow halo, with light orange to cinnamon-red pustules that are smaller, more circular, and more densely packed than common rust; found almost exclusively on upper leaf surface and can also appear on stalk, husk, and leaf sheath.. Pustules almost exclusively on upper leaf surface; smaller, more circular, and more densely packed than common rust; light orange to cinnamon-red urediniospores; black teliospores form in a ring around lesions as the season progresses; can develop on stalk, husk, and leaf sheath in addition to leaves.. Common Rust, Gray Leaf Spot</t>
+          <t>Roots develop small yellow-brown lesions that turn dark brown and are obviously decayed.. Initially, small yellow-brown lesions develop on roots; roots later turn dark brown and are obviously decayed. Fine roots slough off after rotting; their absence is another root rot symptom.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tar_Spot</t>
+          <t>Rhizoctonia</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Phyllachora maydis</t>
+          <t>Rhizoctonia solani</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1890,17 +1834,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Stem, Root, Crown, Foliage</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Yellow to tan flecks on corn leaves, husks, or stalks with black, glossy, raised fungal fruiting bodies (stromata) embedded in host tissue, circular or oval in shape, appearing on both upper and lower leaf surfaces. In severe cases, necrotic halos coalesce causing leaf blight and premature senescence.. Black, glossy, raised fungal fruiting bodies (stromata) that are circular or oval in shape, embedded in host tissue, appearing on both upper and lower leaf surfaces. Raised and black spots cannot be rubbed off with a finger; a necrotic halo may develop around the stromata giving the appearance of a fisheye lesion.. Common Rust, Southern Rust, Physoderma Brown Spot</t>
+          <t>Rhizoctonia causes a variety of symptoms including damping off, stem lesions, stem rot, root rot, crown rot, and aerial web blighting. Infection causes wilting, stunting and possibly plant death.. Girdling lesions at soil line; reddish-brown lesions that can girdle and rot off roots.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -1925,52 +1869,40 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Root, Fruit</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Infected ears show rough, whitish growth with black specks.. Rough, whitish growth with black specks on the ear, distinguishing it from the colored moldy growths of Fusarium and Penicillium.. Nigrospora ear rot</t>
+          <t>Soft, watery rot originating at wounded areas that progresses quickly and can result in full decay of an infected root in as little as three days. Rotted fruit appears slightly darker than brown rot, with skin that may slip away from decaying flesh, and very leaky tissue.. White to grey fungal mycelium producing black sporangia observed growing on decayed roots, resembling a distinctive 'grey man's beard'; skin slipping away from flesh; gray to black fruiting bodies at tips of mycelium whiskers.. brown rot</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Penicillium_On_Seedling</t>
+          <t>Pythium_Diseases</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Penicillium spp.</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Fungal</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Root, Seed, Stem, Foliar</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Discolored and rotted roots and mesocotyl. Blue-green fungal growth on infected seeds. Browning of leaf tips. Entire plants may turn yellow and die or remain discolored and stunted.. Blue-green fungal growth visible on infected seeds; bluish appearance of infected tissue; browning of leaf tips. Entire plants may turn yellow and die.. Pythium seedling blight and root rot, Fusarium seedling blight and root rot, Rhizoctonia seedling blight and root rot</t>
-        </is>
-      </c>
+          <t>Pythium spp.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G45" t="n">
@@ -1980,83 +1912,139 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Anthracnose_Ear_Infection</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
+          <t>Pythium_Stalk_Rot</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Pythium aphanidermatum</t>
+        </is>
+      </c>
       <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Stem</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Pythium stalk rot commonly becomes apparent when the plant suddenly falls over. Diseased areas are dark brown, water-soaked, soft, and collapsed.. Dark brown, water-soaked, soft, and collapsed diseased areas with stalks that may be twisted and distorted; infected plants remain green and turgid for a short time after collapse because the vascular bundles remain intact.</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Chocolate_Spot</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
+          <t>Sugarcane_Mosaic_Virus</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Sugarcane mosaic virus (SCMV), Sorghum mosaic virus (SrMV), Sugarcane streak mosaic virus (SCSMV)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Foliar, Stem, Root, Vascular, Whole plant</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Leaves display irregular yellow and green inlays, stripes, or mottles alternating with parallel veins, ranging from narrow pale-yellow streaks to complete chlorosis, with severely infected leaves turning yellow or yellow-white. Tips of new leaves may become abnormally twisted.. Symptoms are especially visible in the middle and lower sections of new leaves and are more clearly visible when examined against sunlight. Symptoms may be cryptic or indistinct at high temperature but recur when temperature drops.</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Diplodia</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
+          <t>Tar_Spot</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Phyllachora maydis</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Foliar, Stem</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Yellow to tan flecks on corn leaves, husks, or stalks with black, glossy, raised fungal fruiting bodies (stromata). Necrotic halos develop around stromata creating fisheye lesions; in severe cases these coalesce to cause leaf blight and premature senescence.. Black, glossy, raised fungal fruiting bodies (stromata) typically circular or oval in shape, embedded in host tissue, appearing on both upper and lower leaf surfaces. Stromata become visible two to three weeks after infection and are surrounded by a distinctive necrotic halo creating a fisheye lesion appearance.</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ear_Rots</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
+          <t>Bacterial_Leaf_Streak</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Xanthomonas vasicola pv. vasculorum</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Foliar</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>General_And_Mixed_Ear_Rots</t>
+          <t>Anthracnose_Ear_Infection</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -2075,7 +2063,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Genetic_Flecking_Or_Striping</t>
+          <t>Aspergillus_Ear_And_Kernel_Rot</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -2094,7 +2082,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Genetic_Streaking</t>
+          <t>Bacterial_Rot_And_Blight</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -2113,7 +2101,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Leaf_Blight</t>
+          <t>Brown_Spot</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -2132,7 +2120,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Leaf_Spot</t>
+          <t>Charcoal_Stalk_Rot</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -2151,7 +2139,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maize_Lethal_Necrosis</t>
+          <t>Chocolate_Spot</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -2170,7 +2158,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maize_Streak_Virus</t>
+          <t>Cladosporium_Fungus</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -2189,7 +2177,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Rust</t>
+          <t>Corn_Smut</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -2208,7 +2196,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Smut</t>
+          <t>Corn_Stunt_Spiroplasma</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -2227,7 +2215,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Trichoderma_Stalk_Rot</t>
+          <t>Diplodia</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -2243,6 +2231,538 @@
         <v>0</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Diplodia_Stalk_Rot</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Dry_Rot_Of_Ears_And_Stalks_Of_Maize</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Ear_Rots</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Epicoccum_Fungus</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Fusarium_Graminearum_Schwabe</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Fusarium_Wilts</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>General_And_Mixed_Ear_Rots</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>General_And_Mixed_Stalk_Rots</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Genetic_Flecking_Or_Striping</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Genetic_Streaking</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Goss</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Green_Mold</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Khuskia_Fungus</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Leaf_Blight</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Leaf_Spot</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Maize_Lethal_Necrosis</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Maize_Streak_Virus</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Pantoea</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Penicillium_Fungi</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Pythium</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Rust</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Smut</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Southern_Corn_Leaf_Blight_And_Stalk_Rot</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Southern_Corn_Rust</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Stewart_S_Disease</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Trichoderma_Stalk_Rot</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>White_Ear_Rot_And_Seedling_Blight_Of_Maize</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Xanthomonas_Vasicola</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh Corn KB from final-data-update
Replace disease_registry/outputs/Corn/ with the newer version from
origin/final-data-update@cdf1d8da. Adds discovery_results.json,
final_registry.json, raw_extractions.json, registry.md alongside
the updated internet.xlsx (15404 → 15896 bytes).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/disease_registry/outputs/Corn/internet.xlsx
+++ b/disease_registry/outputs/Corn/internet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,12 +456,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Common_Rust</t>
+          <t>Anthracnose_Leaf_Spot_And_Top_Dieback</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Puccinia sorghi</t>
+          <t>Colletotrichum graminicola</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Foliar</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dark, reddish-brown pustules (uredinia) scattered over both upper and lower leaf surfaces, oval to elongate in shape, less than 1/4 inch long, surrounded by broken leaf epidermal layer. Pustules turn brownish-black as plant matures. Under severe conditions, leaf chlorosis and death may occur.. Oval to elongate dark reddish-brown pustules (uredinia) less than 1/4 inch long occurring on both the upper and lower leaf surfaces, surrounded by broken epidermis, distinguishing it from Southern rust which has pustules predominantly on the upper surface. Pustules may develop in bands across the leaf if infection occurs while leaves are in the whorl. Pustules darken to brownish-black as plant matures.. Southern rust</t>
+          <t>Oval or spindle-shaped leaf lesions with tan or brown centers and dark brown or purple margins, up to 1 inch long and ½ inch wide. Lesions can enlarge and join to blight entire leaves. As disease develops, black spiny fruiting structures appear on dead leaf tissue.. Black, spiny fruiting structures visible with a 30X hand lens on dead tissue; oval or spindle-shaped lesions with distinctive dark brown or purple margins.. Gray Leaf Spot, Eye spot</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -485,18 +485,18 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cladosporium_Ear_Rot</t>
+          <t>Anthracnose</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cladosporium herbarum</t>
+          <t>Colletotrichum graminicola</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,12 +506,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Foliar, Stem, Root, Vascular</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Dark green or black powdery mold and black streaks on kernels, with dark green or brown fuzzy mold growing on and between kernels. Mold typically forms first where kernels attach to the cob. Dark kernels scattered around the ear are also observed.. Gray to black or very dark green powdery fungal growth with black streaks in kernels; dark green fuzzy mold between kernels forming first at the kernel-cob attachment point; dark kernels scattered around the ear.</t>
+          <t>Anthracnose manifests in three phases: leaf blight with tan to brown oval lesions and black hair-like fungal structures (setae), top dieback causing stalk death above the ear, and stalk rot with shiny black discoloration and internal decay of pith and vascular tissue. In the leaf blight phase, small round to irregular water-soaked spots first appear on lower leaves, turning yellow then brown with reddish-brown borders.. Black setae (hair-like fungal structures) visible with a hand lens from necrotic leaf lesions; shiny black discoloration in blotches or streaks on lower stalk internodes that cannot be scraped off with a fingernail; shredded pith internally in stalk rot phase.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -520,20 +520,16 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Common_Smut</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Ustilago maydis</t>
-        </is>
-      </c>
+          <t>Alternaria_Black_Molds_Stem_Cankers</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Fungal</t>
@@ -541,17 +537,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Seed</t>
+          <t>Foliar, Stem, Pod</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Galls (abnormal growths) can appear anytime throughout the growing season on any above-ground plant part, including ears, leaves, stalks, or tassels. Galls are initially covered with white to silvery tissue, later developing dark masses of spores inside.. White to silvery galls on ears, leaves, stalks, or tassels that later fill with dark spore masses; leaf galls generally remain small compared to ear and stalk galls.</t>
+          <t>Black molds appear as light to dark brown lesions on the surface of ripe fruits, later covered in a black layer. Cankers appear on stems, leaves, and fruit with dark brown to black color and can lead to plant death.. Lesions vary from small flecks affecting epidermal tissue to large sunken lesions with decay extending into carpel walls. During warm, humid weather, a black velvetlike layer forms on sunken lesions.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -561,62 +557,58 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Anthracnose_Leaf_Spot_And_Top_Dieback</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Colletotrichum graminicola</t>
-        </is>
-      </c>
+          <t>Bacterial_Brown_Spot_Of_Beancanker_Of_Stone_Fruit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Foliar, Pod</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Oval or spindle-shaped tan or brown lesions with dark brown or purple margins (up to 1 inch long and ½ inch wide) beginning on lower leaves and progressing upward; lesions may enlarge up to 5–6 inches, join, and blight entire leaves. Black, spiny fruiting structures develop on dead tissue. Severely infected leaves may yellow and wither.. Black, spiny fruiting structures (acervuli with setae) visible with a 30X hand lens on dead leaf tissue; oval/spindle-shaped lesions with dark brown or purple margins. Resistant lines show only small, necrotic or chlorotic lesions.</t>
+          <t>Small brown spots on leaves that coalesce with yellowing; affected leaves develop a shot-hole appearance. Pods develop water-soaked spots that are sticky with a tiny white crusty center, eventually becoming brown and necrotic.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aspergillus_Ear_Rot</t>
+          <t>Goss_S_Wilt</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aspergillus flavus</t>
+          <t>Clavibacter michiganensis subspecies nebraskensis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Foliar, Stem, Vascular</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Olive-green to gray-green powdery mold on corn kernels, typically starting at the tip of the ear or at insect/bird/hail injury sites; spores disperse like dust when husks are pulled back. Infected kernels may appear discolored and shriveled.. Olive-green (not denim-blue) powdery mold on kernels; signs most commonly at ear tip but can be scattered throughout the ear to the base; spores disperse like dust when husk is pulled back; discolored and shriveled kernels near ear tip are associated with higher aflatoxin levels.. Penicillium ear rot</t>
+          <t>Leaves develop elongated tan lesions with irregular margins and dark water-soaked spots ('freckles'); shiny patches of dried bacterial ooze resembling dry varnish are often present on lesions; infected stalks show orange vascular bundles. Lesions can coalesce to form larger areas.. Shiny patches of dried bacterial ooze resembling dry varnish on leaf lesions; dark green to black discontinuous water-soaked spots ('freckles') within lesion margins that appear as transparent spots when observed against light; elongated tan lesions extending parallel to leaf veins; orange vascular bundles visible in infected stalks.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -631,27 +623,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Diplodia_Ear_Rot</t>
+          <t>Bacterial_Stalk_Rot</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Stenocarpella maydis</t>
+          <t>Erwinia chrysanthemi pv. zeae</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Seed, Pod</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>White fungal mycelium growing over and between kernels starting from the base of the ear. Severely affected ears turn grayish-brown, become lightweight (mummified), with rotted, soft kernels, cobs, and ear leaves. Ear leaves generally die prematurely on infected ears and husks have a bleached appearance.. Raised black bumps (pycnidia) on moldy husk or kernels; 'hidden Diplodia' shows brown kernel discoloration with pycnidia visible only when ear is broken in half. White mycelium growing from base of ear distinguishes Diplodia from Gibberella and Fusarium ear rots.. Gibberella ear rot, Fusarium ear rot</t>
+          <t>Initial discoloration of leaf sheath and stalk at nodes, progressing to lesions on leaves and sheath. Lowest internodes turn tan to brown and become water-soaked, soft, or slimy with foul odor; upper leaves wilt and soft rot occurs at the base of the whorl. The stalk rots completely and the top collapses, causing lodging.. Soft slimy rot mostly initiating at the nodes; splitting the stalk reveals internal discoloration and soft slimy rot; foul odor during decay; water-soaked soft tan-to-brown internodes.. Pythium stalk rot</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -666,12 +658,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fusarium_Disease</t>
+          <t>Aspergillus_Ear_Rot</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Fusarium verticillioides</t>
+          <t>Aspergillus flavus</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -681,12 +673,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Ear, Kernels</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Whitish to pink-colored fungal growth on kernels, often at the ear tip, sometimes with a starburst pattern of white lines radiating from a point on the kernel. Infected kernels may also be scattered on the ear.. Whitish to pink fungal growth at ear tip, and a starburst pattern appearing as white lines radiating out from a point on the kernel. Kernels can also be infected without visible symptoms.. Gibberella ear rot, Diplodia ear rot, Aspergillus ear rot</t>
+          <t>An olive-green to gray-green powdery mold appearing on corn kernels, often beginning at the ear tip and dispersing like dust when husks are pulled back; associated with discolored and shriveled kernels near the tip of the ear.. Distinctive olive-green to gray-green powdery appearance on kernels and ear; fungal spores appear powdery and disperse like dust; signs most commonly at ear tip but can be scattered throughout the ear and to the base; often associated with insect, bird, or hail injury.. Penicillium ear rot</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -695,103 +687,91 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bacterial_Stalk_Rot</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Erwinia chrysanthemi pv. zeae</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Bacterial</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Stem, Foliar, Whole plant</t>
-        </is>
-      </c>
+          <t>Penicillium_Ear_Rot</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Water-soaked, tan to brown, soft and mushy lower internodes causing sudden plant collapse, with vascular strands remaining intact; soft, brown, water-soaked rind and pith; foul odor from infected tissue; stalk twists and falls over while plant may remain green.. Water-soaked lower internodes turning tan to brown, soft and mushy; vascular strands remain intact after collapse; foul odor from infected tissue; decay at first internode above soil; stalk twists and falls over but plant may remain green because vascular tissue is not destroyed; diseased plants scattered throughout field rather than clustered.. Bacterial Top Rot, Fusarium Stalk Rot</t>
+          <t>A powdery denim-blue mold on corn ears.. Denim-blue powdery mold appearance, distinguishing it from the olive-green color of Aspergillus ear rot.. Aspergillus ear rot</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Barley_Yellow_Dwarf_Virus</t>
+          <t>Diplodia_Ear_Rot</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Barley yellow dwarf virus (BYDV)</t>
+          <t>Stenocarpella maydis and Stenocarpella macropora</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Foliar, Whole plant</t>
+          <t>Ear, Kernel, Cob, Husk</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Purpling or yellowing along leaf margins on both lower and upper leaves, with potential stunting, shorter ears, and blanking of tip ends in early infections.. Purpling or yellowing along leaf margins running the full length of leaves; color depends on variety. Distinguished from phosphate deficiency which occurs mainly on young plants.. Phosphate deficiency</t>
+          <t>White mycelium grows over and between kernels, usually starting from the base of the ear. Under highly favorable weather conditions, entire ears may become colonized, turn grayish-brown in color and lightweight (mummified), with kernels, cobs, and ear leaves that are rotted and soft.. White mycelium of the fungus growing over and between kernels, usually starting from the base of the ear — distinguishes Diplodia from Gibberella and Fusarium ear rots. Gibberella ear rot, Fusarium ear rot</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Maize_Dwarf_Mosaic_Virus</t>
+          <t>Fusarium_Disease</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Maize dwarf mosaic virus</t>
+          <t>Fusarium verticillioides</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Seed, Whole plant</t>
+          <t>Kernel, Ear</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Narrow, light green to yellow streaks along leaf veins, leaf sheaths, and husks; plants may be stunted with numerous tillers and poor seed set. Symptoms often begin as chlorotic spots and streaks on young leaves developing into mottle or mosaic patterns, with potential stunting and shortened upper internodes.. Chlorotic spots and streaks on young green leaves progressing to mottle or mosaic pattern; narrow, light green to yellow streaks along leaf veins; mosaic symptoms may disappear as temperature rises while young leaves become more yellow; shortened upper internodes and excessive tillering. Symptoms confined to whorl leaves (unlike Maize white line mosaic virus).. Ear rot, Stalk rot, Maize white line mosaic virus</t>
+          <t>White to salmon-pink discoloration of individual kernels or groups of kernels scattered over the ear. A white to pinkish weft of mycelia covers the kernels, especially on the tip of the ear. White, gray, and pink kernel streaking with starburst patterns may also be observed.. White to salmon-pink discoloration with visible mycelia covering; in severe cases ears are completely consumed, leaving lightweight husks cemented to kernels by mycelia; characteristic starburst symptoms and multi-colored streaking pattern</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -800,33 +780,33 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Corn_Stunt_Spiroplasma</t>
+          <t>Charcoal_Rot</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Spiroplasma kunkelii</t>
+          <t>Macrophomina phaseolina</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Root, Seed, Vascular, Whole plant</t>
+          <t>Root, Stem, Vascular</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Chlorosis and/or reddening of leaf tips, followed by axillary bud production, tillering, severe plant stunting due to shortened internodes, and production of multiple small ears with missing kernels.. Chlorotic stripes extending toward leaf tips, reddening of leaves, severe stunting from shortened internodes, and multiple small ears with missing kernels. Symptoms appear late in season, generally 30 days after leafhopper feeding, during reproductive stages. Severely infected plants may be only 5 feet tall with very short internodes, and stalks may bear multiple ears (up to 6-7) with loose kernels ('loose tooth ears').</t>
+          <t>Charcoal rot begins as a root infection spreading into lower stalk internodes; infected stalks become shredded with completely rotted pith leaving only stringy vascular strands intact; tiny black spherical sclerotia on the vascular strands give the internal stalk tissue a gray/charred appearance; upper leaves dry out; plants wilt.. Small, black, spherical sclerotia of the fungus found on and in vascular strands, numerous enough to give internal stalk tissue a gray color; pith is completely rotted while stringy vascular strands remain more or less intact.. Insufficient water stress, Bacterial wilt, Root problems</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -835,33 +815,33 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Crazy_Top</t>
+          <t>Carbonum_Leaf_Spot</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sclerophthora macrospora</t>
+          <t>Cochliobolus carbonum</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Oomycete</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Whole plant</t>
+          <t>Foliar</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Plants are distorted and/or stunted with a bushy appearance at the top due to leaf proliferation below the tassel, shortened or elongated internodes, excessive tillering, narrow strap-like leaves, and possible lack of ear and tassel formation.. Proliferation of leaves below the tassel giving a very bushy appearance to the top of the plant, excessive tillering, narrow strap-like leaves, and shortened internodes.</t>
+          <t>Symptoms typically appear at silking or full maturity, consisting of circular tan to brown lesions (1/8 to ½ inch) running in a line along the leaf vein.. Lesions arranged in a linear pattern along leaf veins, often described as looking like a 'string of pearls.'</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -876,43 +856,47 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Damping_Off</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t>Barley_Yellow_Dwarf_Virus</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Barley yellow dwarf virus (BYDV)</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Stem, Seed, Whole plant</t>
+          <t>Foliar, Whole plant</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Corn seedlings are stunted compared to healthy seedlings, with a rotted mesocotyl. Affected seedlings occur in areas with heavier, wetter soil.. Rotted mesocotyl on stunted seedlings; the mesocotyl should normally remain firm and white through at least growth stage V6.. Anhydrous ammonia injury, Wireworm damage, Cold injury</t>
+          <t>Symptoms appear as faint yellowish-green blotches near the leaf tip that enlarge and merge, changing to red-purple in oats, yellow-red in wheat, and bright yellow in barley. Infected plants are dwarfed with leaves becoming stiff and erect.. Reddish-purple or yellowish discoloration of the flag leaf combined with plant dwarfing. Symptom color varies by host: red-purple in oats, yellow-red in wheat, bright yellow in barley. Also presents with upright, stiff leaves with serrated edges, reduced tillering and flowering, and sterility with fewer, smaller kernels.. mineral deficiencies, low temperature damage, root rots, herbicide injury</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Diplodia_Stalk_Rot</t>
+          <t>Physoderma_Brown_Spot</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Stenocarpella maydis</t>
+          <t>Physoderma maydis</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -922,47 +906,47 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Stem</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Small black structures embedded within the lower stalk rind, with tan to brown discoloration of macerated pith in lower nodes.. Small black structures embedded within lower stalk rind, distinguishing it from the shiny black areas of anthracnose or the pinhead structures of charcoal rot.. Anthracnose stalk rot, Charcoal rot, Gibberella stalk rot, Fusarium stalk rot</t>
+          <t>Lesions appear on mid-canopy leaves and stalks as dark purple to black discolorations, with banding of yellowish-brown lesions across leaves.. Dark purple to black lesions on stalks and midrib with banding patterns of yellowish-brown lesions across leaves.. Septoria brown spot</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Carbonum_Leaf_Spot</t>
+          <t>Holcus_Spot</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bipolaris zeicola</t>
+          <t>Pseudomonas syringae pv. syringae</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Foliar, Leaf sheath, Husk</t>
+          <t>Foliar</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Circular tan to brown lesions (1/8 to 1/2 inch) running in a line along the leaf vein, often described as looking like a "string of pearls." Also described as grayish tan lesions surrounded by a darker border on lower leaf blades, narrow and up to 1 inch long. Symptoms usually appear at the time of silking or full maturity.. Circular tan to brown lesions arranged in a line along the leaf vein, resembling a "string of pearls". Race 2 produces oblong lesions mainly on lower leaves and on maturing plants. Race 3 produces narrow, linear lesions on leaves, leaf sheaths, and sometimes husks.. Northern Corn Leaf Blight, Southern Corn Leaf Blight, Anthracnose, Gray Leaf Spot</t>
+          <t>Water-soaked, dark green lesions initially appear near leaf tips, developing into round or elliptical tan to white spots with red to brown margins and yellow halos.. Round or elliptical tan to white spots 1/8 to 1/4 inch in diameter with red to brown margins that may be surrounded by yellow halos; spots lack margins typical of eyespot and do not necessarily develop on lower leaves first.. Paraquat damage, eyespot, gray leaf spot</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -971,18 +955,18 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Gibberella_Disease</t>
+          <t>Cladosporium_Ear_Rot</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fusarium graminearum</t>
+          <t>Cladosporium herbarum</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -997,27 +981,27 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Red or pink colored mold on corn ears, almost always beginning at the tip of the ear. In severe cases, pink mold is visible on the outside of the husks at the ear tip. Excessive mold may cause silks and husks to adhere to the ear.. Red or pink mold starting at the ear tip; infection via the silk channel; excessive mold causing silks and husks to adhere to the ear; pinkish-white mold at the tip.. Fusarium Kernel or Ear Rot</t>
+          <t>Dark (brown to green) fuzzy mold grows on and between kernels, with dark kernels scattered around the ear.. Gray to black or very dark green fungus with a powdery appearance; also causes black streaks in the kernels.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nigrospora_Ear_Rot</t>
+          <t>Common_Rust</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nigrospora oryzae</t>
+          <t>Puccinia sorghi</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1027,32 +1011,32 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Gray fungal growth on corn kernels with small black spores. Corn cobs prone to shredding during shelling.. Small black spores that can be removed by rubbing with a finger, unlike the pycnidia of Diplodia ear rot. Gray fungal growth on kernels.. Diplodia Ear Rot</t>
+          <t>Common rust begins with small tan spots on leaves with a characteristic yellow halo, progressing to brick-red to cinnamon-brown pustules that readily rub off onto fingers.. Characteristic yellow halo with jagged, elongate, brick-red to cinnamon-brown pustules that readily rub off; as disease progresses, darker orange-brown teliospores create darker pustules.. Gray leaf spot</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Penicillium_Ear_Rot</t>
+          <t>Eyespot</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Penicillium spp.</t>
+          <t>Aureobasidium zeae (synonym: Kabatiella zeae)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1062,12 +1046,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Kernel, Ear tip</t>
+          <t>Leaf, Leaf sheath, Husk</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Green or blue-green powdery mold growing between kernels, usually at the tip of the ear. Infected kernels can appear bleached or streaked.. Green or blue-green powdery mold between kernels, typically at ear tip; bleached or streaked kernels; 'blue-eye' condition (embryo discoloration) in stored grain at high moisture.</t>
+          <t>Initial symptoms are small, circular water-soaked or chlorotic spots (1/16 to 1/8 inch diameter) with yellow halos. The center tissue dies and turns tan-colored with a brown to purple ring at the margin. The yellow halo is clearly visible when the leaf is lighted from behind. Spots may coalesce into large necrotic areas and entire leaves may die.. Yellow halo clearly visible when the leaf is lighted from behind, surrounding a tan-colored necrotic center with a brown ring at the margin. Physiological leaf spot, Genetic leaf spot</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1082,47 +1066,35 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Trichoderma_Ear_Rot</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Trichoderma afroharzianum</t>
-        </is>
-      </c>
+          <t>Gray_Leaf_Spot</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>Fungal</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Seed, Husk</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>White mycelium growing between kernels and on husk leaves, with massive production of green to gray-green conidia, often covering the entire ear and causing premature ripening of kernels. Kernels may sprout on the cob if disease is severe.. Dark blue-green layers of conidia on and between kernels; white mycelium on husk leaves turning green to gray-green; premature germination/ripening of kernels; symptoms typically occurring from base to middle of cob covering all kernels and husk leaf layers.. Fusarium ear rot</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Charcoal_Stalk_Rot</t>
+          <t>Crown_Rot</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Macrophomina phaseolina</t>
+          <t>Alternaria linariae</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1132,17 +1104,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Root, Stem, Vascular</t>
+          <t>Stem</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Shredded stalks with rotted pith leaving only stringy vascular strands, covered in tiny black spherical sclerotia that give the internal stalk tissue a grey or charred appearance. Upper leaves dry out and plants ripen prematurely.. Very tiny black sclerotia on the vascular strands of the shredded pith giving a charred appearance inside the stalk. This charring of the interior is the distinguishing characteristic.. Diplodia Stalk Rot, Gibberella Stalk Rot</t>
+          <t>In seedlings, collar rot stem lesions are small, dark, and slightly sunken, forming circular or elongated lesions with or without pronounced concentric rings and light centers. Once planted in the field, lesions enlarge around the stem and girdle plants, often causing plant death or severe reduction in growth and yield.. Concentric rings may not always be pronounced, in contrast to Alternaria stem canker which always displays pronounced concentric rings.. Alternaria stem canker</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1152,12 +1124,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Northern_Leaf_Blight</t>
+          <t>Gibberella_Disease</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Exserohilum turcicum</t>
+          <t>Fusarium graminearum</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1167,12 +1139,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Foliar</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Canoe- or cigar-shaped tan to gray lesions 1 to 6 inches long on leaves, initially bordered by gray-green margins. Early lesions appear as small light-green to grayish spots. As disease develops, lesions produce dark gray spores giving a dirty appearance. Severely affected leaves become grayish-green and brittle.. Cigar- or canoe-shaped gray to tan lesions 1–6 inches long; early lesions appear as small light-green to grayish spots 1–2 weeks after infection; mature lesions produce dark gray spores giving a dirty appearance; severely affected leaves become grayish-green and brittle, resembling frost-killed leaves.. Goss's leaf blight, Stewart's wilt</t>
+          <t>GER is characterized by a pink to reddish mold that appears at the tip and grows down the ear. In early ear infection by the disease the entire ear may rot and be covered with a pinkish mycelium that causes the husk to tightly adhere to the ear. Also called red rot, infection is characterized by reddish-pinkish color of infected ears.. Pink to reddish mold progressing from tip down the ear; pinkish mycelium covering the ear causing husk to adhere tightly; blue or black perithecia may cover husk and ear shanks; pinkish-whitish mycelia visible on infected kernels.. Fusarium ear rot</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1181,18 +1153,18 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gray_Leaf_Spot</t>
+          <t>Trichoderma_Ear_Rot</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cercospora zeae-maydis</t>
+          <t>Trichoderma viride</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1202,17 +1174,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Seed, Pod</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Rectangular tan to brown lesions bordered by leaf veins, initially yellow to tan with a faint watery halo, later developing a silvery-gray cast when conidia are produced.. Rectangular lesions bordered by leaf veins, 3 to 4 inches long and 1/16 to 1/8 inch wide, with a silvery-gray cast during sporulation. Early lesions have a faint watery halo visible when held to light.. Anthracnose leaf blight, Bacterial leaf streak, Common rust, Curvularia leaf spot, Eyespot of Corn, Northern corn leaf blight, Southern corn leaf blight</t>
+          <t>Dark green mold growing on or between kernels, often covering the entire ear. Kernels may sprout on the cob if disease is severe.. Dark green mold appearing on or between kernels and covering the entire ear.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1222,27 +1194,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Downy_Mildew</t>
+          <t>Southern_Rust</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Peronosclerospora sorghi</t>
+          <t>Puccinia polysora</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Oomycete</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Foliar, Whole plant, Seed</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Leaves show yellow to white stripes from base toward tip; plants may be stunted, chlorotic, with irregular seed set. Infected leaves are narrower than usual, erect, and shredded.. Yellow to white striping on leaves from base toward tip, leaves narrower than usual, erect and shredded, white downy mycelium on both leaf surfaces.</t>
+          <t>Southern corn rust begins with small circular-to-oval lesions with light green to yellow halos, developing into light orange to cinnamon-red pustules that are smaller, more circular, and more densely packed than common rust pustules.. Smaller and more circular pustules that are densely packed; almost exclusively located on upper leaf surface; can also develop on stalk, husk, and leaf sheath unlike common rust.. Gray leaf spot</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1257,12 +1229,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Eyespot</t>
+          <t>Common_Smut</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aureobasidium zeae</t>
+          <t>Ustilago maydis</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1272,32 +1244,32 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Foliar</t>
+          <t>Foliar, Stem, Pod</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Small circular water-soaked spots with yellow halos on leaves that develop into tan spots surrounded by brown to purple rings with narrow yellow halos. Spots can join together to form large necrotic areas.. Tan spot surrounded by a brown to purple ring and narrow yellow halo, forming a characteristic 'eyespot' pattern. Lesions can also develop on leaf sheaths and husks.. physiological leaf spot, genetic leaf spot</t>
+          <t>Common smut causes yellowing of green tissue and production of light green or white to gray, fleshy galls on leaves, tassels, stalks and ears, ranging from 0.2 inches on leaves to up to 6 inches on stalks and ears. Galls are filled with black, powdery teliospores that are released when galls rupture.. Galls filled with black, powdery teliospores that rupture to release spores; galls appear light green or white to gray and fleshy; lumpy and mushroom-like in appearance with off-white to grey color, filling with fine black spores.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Crown_Rot</t>
+          <t>Head_Smut</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fusarium spp.</t>
+          <t>Sporisorium reilianum</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1307,12 +1279,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Root, Stem, Foliar, Whole plant</t>
+          <t>Tassel, Ear, Leaf, Vascular</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Stunted, wilted plants with yellowed lower leaves; brown to black discoloration of crown tissue and roots; premature senescence with grayish-green discoloration ('ghost' plants); pinkish or reddish brace roots. Stalk nodes appear reddish-brown to dark black; leaf firing starts from plant base and progresses upward.. Dark brown to black discoloration of crown interior and roots; stalk nodes rot progressively up the stalk but internodes are not typically symptomatic; distinguishable from red root rot by dark brown-black (vs. deep red-purple) discoloration. Dark discoloration visible as early as 2-leaf stage.. Red root rot, Fusarium stalk rot, Root rot</t>
+          <t>Head smut is characterized by large smut galls that replace ears or tassels, first covered by fragile, creamy white membranes that eventually rupture to release masses of dark brown spores. Sporulating fungal sites may also appear on leaves, with coarse galls revealing dry spore masses with visible strands of vascular tissue.. The vascular bundles within the galls readily differentiate head smut from common smut, giving the spore masses a stringy appearance. The gall is coarse and on eruption reveals dry spore masses with strands of vascular tissue.. common smut</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1327,49 +1299,45 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rhizoctonia</t>
+          <t>Crazy_Top</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rhizoctonia solani</t>
+          <t>Sclerophthora macrospora</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Oomycete</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Root, Stem, Whole plant</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Reddish-brown lesions on the lower stem at soil level. In corn, seedlings may die and rot below the soil surface, characterized by water-soaked and dark mesocotyl tissue that can be removed to reveal white inner vascular tissue. Also causes damping off, stem rot, root rot, crown rot, aerial web blighting, wilting, and stunting.. Reddish-brown lesions on the lower stem at soil level; in corn, water-soaked dark mesocotyl tissue removable to reveal white inner vascular tissue; girdling lesions at the soil line; small brown sclerotia may be present.. Pythium seedling disease, Fusarium root rot, Phytophthora root rot</t>
+          <t>The disease causes proliferation of the tassel where leafy structures develop instead of a normal tassel, along with abnormal tillers and chlorotic striping on leaves.. Proliferation of the tassel with a mass of leafy structures developing instead of a normal tassel structure.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Physoderma_Brown_Spot</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Physoderma maydis</t>
-        </is>
-      </c>
+          <t>Damping_Off</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Fungal</t>
@@ -1377,74 +1345,82 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Numerous very small round or oval yellowish to brown spots occurring in broad bands across the leaf, with dark purplish to black oval spots on the midrib, stalk, leaf sheath, and husks. As disease progresses, lesions coalesce and darken to chocolate, reddish brown, or purple.. Lesions develop in distinct bands across the leaf, particularly at the base. On the leaf midrib, lesions are darker and sometimes larger. Purplish to black oval spots on the midrib are filled with thousands of sporangia. Lesions are not rust pustules under magnification.. Southern Rust, Eyespot, Purple leaf sheath</t>
+          <t>Diseased corn seedlings are stunted with a rotted mesocotyl.. A rotted mesocotyl where it should normally remain firm and white.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>General_And_Mixed_Stalk_Rots</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
+          <t>Downy_Mildew</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Peronosporaceae spp. (oomycetes)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Oomycete</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Stem, Vascular</t>
+          <t>Foliar, Stem, Root, Seed, Whole plant</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Weakened stalks that are susceptible to lodging before harvest, with reduced ability to transport water and nutrients.</t>
+          <t>Characteristic symptoms include development of chlorotic streaks on leaves with stunted and bushy plant appearance due to shortened internodes, and white downy growth visible on the lower leaf surface.. White downy growth on the lower surface of leaves consisting of sporangiophores bearing hyaline, oblong or ovoid sporangia; downy growth also appears on bracts of unopened male flowers in the tassel; proliferation of axillary buds on stalk and cobs.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pythium_Stalk_Rot</t>
+          <t>Northern_Leaf_Blight</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pythium aphanidermatum</t>
+          <t>Exserohilum turcicum</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Oomycete</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Stem</t>
+          <t>Foliar, Leaf sheaths, Ear husks</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Plants suddenly fall over with dark brown, water-soaked, soft, and collapsed areas on a single internode near the soil line. The rind and pith become soft, brown, and water-soaked. Stalks may be twisted and distorted, but plants remain green and turgid briefly after collapse because the vascular tissue is not destroyed.. Infected plants remain green and turgid for a short time after collapse because the vascular bundles remain intact, distinguishing it from other stalk rots where wilting occurs simultaneously. Decay localized to the first internode above the soil; rind and pith become soft, brown, and water-soaked; stalk twists and falls over.. Anthracnose Stalk Rot, Bacterial Stalk Rot, Diplodia Stalk Rot, Fusarium Stalk Rot, Gibberella Crown Rot and Stalk Rot, Physoderma Stalk Rot</t>
+          <t>Characteristic cigar-shaped gray- to tan-colored lesions on corn leaves that initially appear as small light-green to grayish spots and develop dark gray spores, eventually destroying leaves and causing them to become grayish-green and brittle. Early symptoms appear as long, narrow tan lesions running parallel to leaf veins that expand to form long, oblong, or cigar-shaped tan to gray lesions.. One-to-six inch long cigar-shaped gray to tan lesions; compatible interactions produce large necrotic cigar-shaped lesions while incompatible interactions produce small chlorotic lesions. Lesions eventually coalesce and may cover a significant portion of the leaf, with small fungal spores appearing as tiny black or dark green specks inside lesions when observed with a hand lens.. Gray leaf spot</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1459,62 +1435,62 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Head_Smut</t>
+          <t>Maize_Chlorotic_Dwarf_Virus</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sphacelotheca reiliana</t>
+          <t>Maize chlorotic dwarf virus</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Tassel, Ear, Whole plant</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Large smut galls replace ears or tassels, first covered by fragile creamy white membranes that rupture to release masses of dark brown spores. Leaf-like proliferations develop on tassels and ears; infected ears are teardrop-shaped and lack silks. Plants may be severely dwarfed.. Intact threadlike strands of vascular bundles within spore masses give a stringy appearance, differentiating head smut from common smut. Teardrop-shaped ears lacking silks with husks filled with teliospores. Plants are systemically infected as seedlings though symptoms are only obvious at flowering.. Common smut</t>
+          <t>MCDV causes plant stunting, leaf reddening or yellowing, leaf twisting and tearing, and chlorosis of leaf veins (vein banding). Infected leaves may develop a rough corduroy texture.. Vein banding (chlorosis of leaf veins) is the most diagnostic symptom. Infected leaves develop a rough corduroy texture instead of smooth and shiny appearance.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Southern_Corn_Leaf_Blight</t>
+          <t>Maize_Dwarf_Mosaic_Virus</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Bipolaris maydis</t>
+          <t>Maize dwarf mosaic virus</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Seed</t>
+          <t>Foliar, Stem, Whole plant</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tan, rectangular lesions with reddish-brown margins on leaves (Race O); rectangular to elliptical lesions with reddish-brown border and chlorotic zone on leaves, purple spots with tan-gray centers on stalks, and gray-black felt-like mold on ears (Race T).. Rectangular spots confined by leaf veins, light brown with darker brown margin, starting on lower leaves, oval at first becoming rectangular up to 2.5 cm long and 2-6 mm wide; Race T lesions rectangular to elliptical with reddish-brown border surrounded by a chlorotic zone; stalk infections as purple spots developing tan-gray centers; ear infections as gray-black felt-like mold extending from husk into kernels.</t>
+          <t>Symptoms include narrow, light green to yellow streaks along veins of leaves and husks that may disappear with temperature rise, while young leaves become more yellow. Symptoms often begin as chlorotic spots and streaks on young leaves developing into a mottle or mosaic pattern. Plants may be stunted with numerous tillers and poor seed set.. Narrow, light green to yellow streaks along leaf veins and husks transitioning to yellow leaves as temperature increases; chlorotic spots and streaks on young leaves progressing to mosaic or mottle pattern; shortened upper internodes; excessive tillering.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1529,62 +1505,54 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Holcus_Spot</t>
+          <t>Maize_White_Line_Mosaic</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pseudomonas syringae pv. syringae</t>
+          <t>Aureusvirus zeae</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bacterial</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Foliar</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Circular, oval, or irregular dark green water-soaked spots that dry to light tan or white with papery texture, often developing light brown to reddish margins surrounded by yellow halos. Spots range from 1/8 to 1/4 inch in diameter and appear randomly across the leaf surface, especially on the upper half of leaves and near tips of lower leaves.. Spots are larger than a pencil eraser tip, lesion patterns vary leaf to leaf, water-soaked margins are present, and symptoms do not follow a clear gradient across the field. Lesions are randomly distributed with tan centers and reddish-brown margins or yellow halos. Round or elliptical tan to white spots 1/8 to 1/4 inch in diameter with red to brown margins and yellow halos.. Contact herbicide injury (paraquat), Eyespot, Gray Leaf Spot, Tar Spot</t>
-        </is>
-      </c>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Goss_S_Wilt</t>
+          <t>Nigrospora_Ear_Rot</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Clavibacter michiganensis subsp. nebraskensis</t>
+          <t>Nigrospora oryzae</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Foliar, Vascular, Stem, Whole plant</t>
+          <t>Seed, Cob</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Long, gray-green to black, water-soaked leaf lesions with wavy edges containing distinctive dark freckle-like streaks; bacterial exudate droplets dry into crystalline deposits on the leaf surface. Systemically infected plants may show discolored vascular tissue and slimy stalk rot.. Dark freckle-like streaks within lesions that are transparent when held to light, with crystalline deposits from dried bacterial exudate on the leaf surface. Lesions have distinctive wavy edges. Freckles appear as dark green to black discontinuous water-soaked spots near the edges of expanding lesions.</t>
+          <t>Nigrospora ear and cob rot displays dark gray or black fungal mold and small black spores on kernels, which become bleached with white streaks, while cobs develop a brown tattered appearance and infected ears become lighter with loose kernels. Symptoms are not usually evident until harvest; affected ears are lightweight with the cob shredding easily.. Dark gray or black mold is characteristic of this disease; numerous round black spores form at the tip end of the ear; cob shreds easily, usually at the base of the ear.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1599,97 +1567,97 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Root_Rot</t>
+          <t>Stewart_S_Wilt</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fusarium spp.</t>
+          <t>Pantoea stewartii subsp. stewartii</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Root</t>
+          <t>Foliar, Vascular, Stem, Whole plant</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Dark brown to black, discolored decaying or completely rotted roots.. Dark brown to black discolored decaying or completely rotted roots with complex symptoms.</t>
+          <t>Stewart's wilt exhibits two phases: a seedling wilt phase with water-soaked lesions and rapid wilting, and a leaf blight phase with long linear yellow-grey streaks with wavy margins running parallel to leaf veins, later turning necrotic and dark. Gray-green to yellow-green lesions may cause entire leaves to become straw-colored and necrotic.. Long linear yellow-grey lesions with wavy margins running parallel to leaf veins; water-soaked lesions progressing to necrosis; yellow bacterial slime exuding from vascular bundles in cross-sectional stem cuts; distinct wilt vs. leaf blight phase depending on plant developmental stage at infection.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Maize_Chlorotic_Dwarf_Virus</t>
+          <t>Penicillium_On_Seedling</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Maize chlorotic dwarf virus</t>
+          <t>Penicillium spp.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Foliar, Whole plant</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Plant stunting with shortening of upper internodes, leaf reddening or yellowing, leaf twisting and tearing, chlorosis of leaf veins (vein banding), and a rough "corduroy" texture on infected leaves.. Vein banding (chlorosis or clearing of the smallest visible leaf veins) is the most diagnostic symptom. Leaves may also develop a rough "corduroy" texture instead of being smooth and shiny.. Maize Dwarf Mosaic Virus</t>
+          <t>Seedlings become blighted one to two weeks after emergence with marginal scorching and dying. Green fungal growth is visible in the hypocotyl area immediately above the seed.. Green fungal growth associated with rotted areas on the hypocotyl immediately above the seed.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Maize_White_Line_Mosaic</t>
+          <t>Physoderma_Stalk_Rot</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Maize white line mosaic virus</t>
+          <t>Physoderma maydis</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Foliar, Root, Seed, Whole plant</t>
+          <t>Stem</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Severely stunted plants with bright mosaic on leaves consisting of white, yellow and yellow-green rectangular to linear patches and stripes. Cobs do not fill out, are mis-shapen and contain few kernels.. Symptoms are not confined to whorl leaves (unlike Maize dwarf mosaic virus) but are present in all leaves and persist after pollination. White line and mosaic patterns with rectangular to linear (1-2 cm) patches are distinctive. No other virus known in maize gives symptoms like those of Maize white line mosaic virus.. Maize dwarf mosaic virus</t>
+          <t>Symptoms appear when plants break at the first or second node, which becomes black with some pith rot. Infected nodes snap easily when gently pushed.. Microscopic examination reveals thousands of light brown sporangia where spore production and storage occurs. Infected nodes snap easily when gently pushed.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1704,183 +1672,159 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Physoderma_Stalk_Rot</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Physoderma maydis</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Fungal</t>
-        </is>
-      </c>
+          <t>Purple_Leaf_Sheath</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Stem</t>
+          <t>Foliar, Stem</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Plants break at the first or second node, with black nodes and pith rot present. Infected nodes snap easily if gently pushed. Affected plants often look healthy with no visible brown spot symptoms on leaves.. Black nodes at first or second node, pith rot, nodes that snap easily when pushed, and microscopic light brown sporangia in symptomatic tissue. Brown spot symptoms often are not visible on the leaves of affected plants.. Anthracnose Stalk Rot of Corn, Fusarium Stalk Rot of Corn, Pythium Stalk Rot of Corn, Gibberella Crown Rot and Stalk Rot of Corn, Bacterial Stalk Rot of Corn, Diplodia Stalk Rot of Corn</t>
+          <t>Dark lesions on corn stalks and leaf collars that vary in color from purple to brown to black, typically appearing after the VT tasseling stage.. Lesions appear scattered and random across plants, with tassel debris typically present in the leaf collar area where symptoms develop.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Purple_Leaf_Sheath</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
+          <t>Pythium_Root_And_Stem_Rot</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Pythium spp.</t>
+        </is>
+      </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Abiotic</t>
+          <t>Oomycete</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Stem, Foliar</t>
+          <t>Seed, Root, Stem</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Dark lesions on corn stalks and leaf collars, with color varying from purple to brown to black. Affected plants are scattered and random throughout the field.. Pieces of tassel debris fallen into the leaf collar are present in almost all cases where symptoms appear; lesions are not specific to any hybrid, canopy position, or field location and affected plants are scattered randomly.</t>
+          <t>Symptoms range from stunted, slower-growing plants to severely infected, dead plants, with brown, rotted roots and necrotic mesocotyl. Typical symptoms include seed decay, pre-emergent seedling rot, and seedling damping off. If the plant has emerged, the root system's outer layer can be easily pulled off while the center stays intact; dark lesions may develop on the mesocotyl or root system in corn.. Root system where the outer layer can be easily pulled off with the center remaining intact (rat tail-like appearance); dark lesions on mesocotyl or root system in corn; brown rotted roots and mesocotyl.. Rhizoctonia Root Rot, Fusarium Root Rot, Phytophthora, Insect injury, Herbicide damage</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pythium</t>
+          <t>Common_Corn_Rust</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Pythium spp.</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Oomycete</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Root, Seed, Stem</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Dark, slimy, water-soaked lesions on roots and mesocotyl that cause shriveling. The outer cortex of the root may rot while the inner stele remains white and intact.. Water-soaked appearance of infected tissue; outer root cortex rots while the inner stele remains white and intact; dark, slimy lesions on root or mesocotyl. Most favored by wet/saturated soil conditions due to production of motile swimming zoospores.. Fusarium seedling blight and root rot, Rhizoctonia seedling blight and root rot, Penicillium seedling blight</t>
-        </is>
-      </c>
+          <t>Puccinia polysora</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Stewart_S_Disease</t>
+          <t>Southern_Corn_Leaf_Blight</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pantoea stewartii</t>
+          <t>Bipolaris maydis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Fungal</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Foliar, Vascular, Stem, Whole plant</t>
+          <t>Foliar, Stem, Pod, Seed</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Bleached leaf streaks running the length of the leaf in early phase, progressing to leaf blight after tasseling; internal vascular discoloration and bacterial oozing from cut stems; seedlings may wilt and die when severe.. Bleached leaf streaks that may run the full length of the leaf; bacterial oozing from cut stem cross sections; discoloration of vascular tissues; two distinct phases with early seedling wilt and later leaf blight after tasseling.. Goss's Wilt</t>
+          <t>Two races cause distinct lesion patterns. Race O produces tan lesions with reddish-brown margins on leaves; Race T produces reddish-brown margined lesions with possible chlorotic zones. Stalk infections show purple spots with tan-gray centers, and ear infections display gray-black lesions extending into kernels with black felt-like mold.. Race O distinctly produces tan lesions with reddish-brown margins and rectangular shape; Race T produces reddish-brown margined lesions rectangular to elliptical in shape (1/4 to 1/2 inch wide by 1/4 to 3/4 inch long) possibly surrounded by a chlorotic zone. Stalk infections appear as purple spots developing tan-gray centers. Ear infections show gray-black lesions with black felt-like mold extending into kernels.. Northern corn leaf blight, Northern corn leaf spot</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Southern_Rust</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Puccinia polysora</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Fungal</t>
-        </is>
-      </c>
+          <t>Root_Rot</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Root</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Small circular-to-oval shaped lesions with light green to yellow halo, with light orange to cinnamon-red pustules that are smaller, more circular, and more densely packed than common rust; found almost exclusively on upper leaf surface and can also appear on stalk, husk, and leaf sheath.. Pustules almost exclusively on upper leaf surface; smaller, more circular, and more densely packed than common rust; light orange to cinnamon-red urediniospores; black teliospores form in a ring around lesions as the season progresses; can develop on stalk, husk, and leaf sheath in addition to leaves.. Common Rust, Gray Leaf Spot</t>
+          <t>Roots develop small yellow-brown lesions that turn dark brown and are obviously decayed.. Initially, small yellow-brown lesions develop on roots; roots later turn dark brown and are obviously decayed. Fine roots slough off after rotting; their absence is another root rot symptom.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tar_Spot</t>
+          <t>Rhizoctonia</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Phyllachora maydis</t>
+          <t>Rhizoctonia solani</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1890,17 +1834,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Stem, Root, Crown, Foliage</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Yellow to tan flecks on corn leaves, husks, or stalks with black, glossy, raised fungal fruiting bodies (stromata) embedded in host tissue, circular or oval in shape, appearing on both upper and lower leaf surfaces. In severe cases, necrotic halos coalesce causing leaf blight and premature senescence.. Black, glossy, raised fungal fruiting bodies (stromata) that are circular or oval in shape, embedded in host tissue, appearing on both upper and lower leaf surfaces. Raised and black spots cannot be rubbed off with a finger; a necrotic halo may develop around the stromata giving the appearance of a fisheye lesion.. Common Rust, Southern Rust, Physoderma Brown Spot</t>
+          <t>Rhizoctonia causes a variety of symptoms including damping off, stem lesions, stem rot, root rot, crown rot, and aerial web blighting. Infection causes wilting, stunting and possibly plant death.. Girdling lesions at soil line; reddish-brown lesions that can girdle and rot off roots.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -1925,52 +1869,40 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Root, Fruit</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Infected ears show rough, whitish growth with black specks.. Rough, whitish growth with black specks on the ear, distinguishing it from the colored moldy growths of Fusarium and Penicillium.. Nigrospora ear rot</t>
+          <t>Soft, watery rot originating at wounded areas that progresses quickly and can result in full decay of an infected root in as little as three days. Rotted fruit appears slightly darker than brown rot, with skin that may slip away from decaying flesh, and very leaky tissue.. White to grey fungal mycelium producing black sporangia observed growing on decayed roots, resembling a distinctive 'grey man's beard'; skin slipping away from flesh; gray to black fruiting bodies at tips of mycelium whiskers.. brown rot</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Penicillium_On_Seedling</t>
+          <t>Pythium_Diseases</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Penicillium spp.</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Fungal</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Root, Seed, Stem, Foliar</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Discolored and rotted roots and mesocotyl. Blue-green fungal growth on infected seeds. Browning of leaf tips. Entire plants may turn yellow and die or remain discolored and stunted.. Blue-green fungal growth visible on infected seeds; bluish appearance of infected tissue; browning of leaf tips. Entire plants may turn yellow and die.. Pythium seedling blight and root rot, Fusarium seedling blight and root rot, Rhizoctonia seedling blight and root rot</t>
-        </is>
-      </c>
+          <t>Pythium spp.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G45" t="n">
@@ -1980,83 +1912,139 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Anthracnose_Ear_Infection</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
+          <t>Pythium_Stalk_Rot</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Pythium aphanidermatum</t>
+        </is>
+      </c>
       <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Stem</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Pythium stalk rot commonly becomes apparent when the plant suddenly falls over. Diseased areas are dark brown, water-soaked, soft, and collapsed.. Dark brown, water-soaked, soft, and collapsed diseased areas with stalks that may be twisted and distorted; infected plants remain green and turgid for a short time after collapse because the vascular bundles remain intact.</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Chocolate_Spot</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
+          <t>Sugarcane_Mosaic_Virus</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Sugarcane mosaic virus (SCMV), Sorghum mosaic virus (SrMV), Sugarcane streak mosaic virus (SCSMV)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Foliar, Stem, Root, Vascular, Whole plant</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Leaves display irregular yellow and green inlays, stripes, or mottles alternating with parallel veins, ranging from narrow pale-yellow streaks to complete chlorosis, with severely infected leaves turning yellow or yellow-white. Tips of new leaves may become abnormally twisted.. Symptoms are especially visible in the middle and lower sections of new leaves and are more clearly visible when examined against sunlight. Symptoms may be cryptic or indistinct at high temperature but recur when temperature drops.</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Diplodia</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
+          <t>Tar_Spot</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Phyllachora maydis</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Foliar, Stem</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Yellow to tan flecks on corn leaves, husks, or stalks with black, glossy, raised fungal fruiting bodies (stromata). Necrotic halos develop around stromata creating fisheye lesions; in severe cases these coalesce to cause leaf blight and premature senescence.. Black, glossy, raised fungal fruiting bodies (stromata) typically circular or oval in shape, embedded in host tissue, appearing on both upper and lower leaf surfaces. Stromata become visible two to three weeks after infection and are surrounded by a distinctive necrotic halo creating a fisheye lesion appearance.</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ear_Rots</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
+          <t>Bacterial_Leaf_Streak</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Xanthomonas vasicola pv. vasculorum</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Foliar</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>General_And_Mixed_Ear_Rots</t>
+          <t>Anthracnose_Ear_Infection</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -2075,7 +2063,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Genetic_Flecking_Or_Striping</t>
+          <t>Aspergillus_Ear_And_Kernel_Rot</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -2094,7 +2082,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Genetic_Streaking</t>
+          <t>Bacterial_Rot_And_Blight</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -2113,7 +2101,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Leaf_Blight</t>
+          <t>Brown_Spot</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -2132,7 +2120,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Leaf_Spot</t>
+          <t>Charcoal_Stalk_Rot</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -2151,7 +2139,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maize_Lethal_Necrosis</t>
+          <t>Chocolate_Spot</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -2170,7 +2158,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maize_Streak_Virus</t>
+          <t>Cladosporium_Fungus</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -2189,7 +2177,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Rust</t>
+          <t>Corn_Smut</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -2208,7 +2196,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Smut</t>
+          <t>Corn_Stunt_Spiroplasma</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -2227,7 +2215,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Trichoderma_Stalk_Rot</t>
+          <t>Diplodia</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -2243,6 +2231,538 @@
         <v>0</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Diplodia_Stalk_Rot</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Dry_Rot_Of_Ears_And_Stalks_Of_Maize</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Ear_Rots</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Epicoccum_Fungus</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Fusarium_Graminearum_Schwabe</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Fusarium_Wilts</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>General_And_Mixed_Ear_Rots</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>General_And_Mixed_Stalk_Rots</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Genetic_Flecking_Or_Striping</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Genetic_Streaking</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Goss</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Green_Mold</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Khuskia_Fungus</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Leaf_Blight</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Leaf_Spot</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Maize_Lethal_Necrosis</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Maize_Streak_Virus</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Pantoea</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Penicillium_Fungi</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Pythium</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Rust</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Smut</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Southern_Corn_Leaf_Blight_And_Stalk_Rot</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Southern_Corn_Rust</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Stewart_S_Disease</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Trichoderma_Stalk_Rot</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>White_Ear_Rot_And_Seedling_Blight_Of_Maize</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Xanthomonas_Vasicola</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>